<commit_message>
HQ LAN oldali konfig elkeszult
router:
ip cimek, vlanok, dhcp szerverek
switchek: mgmt ip, vlanok
vegponti eszkozok: fix IP illetve DHCP konfig

HQ eszkozkonfig parancsok rtf-be mentve

IP terv pontositva
</commit_message>
<xml_diff>
--- a/IP terv.xlsx
+++ b/IP terv.xlsx
@@ -28,6 +28,9 @@
     <t>R1</t>
   </si>
   <si>
+    <t>G0/0</t>
+  </si>
+  <si>
     <t>192.168.11.1</t>
   </si>
   <si>
@@ -64,10 +67,13 @@
     <t>192.168.12.11-100</t>
   </si>
   <si>
+    <t>G0/1</t>
+  </si>
+  <si>
     <t>192.168.12.1</t>
   </si>
   <si>
-    <t>SW12-VLAN12</t>
+    <t>SW12</t>
   </si>
   <si>
     <t>192.168.12.2</t>
@@ -98,12 +104,6 @@
   </si>
   <si>
     <t>192.168.13.1</t>
-  </si>
-  <si>
-    <t>SW12-VLAN13</t>
-  </si>
-  <si>
-    <t>192.168.13.2</t>
   </si>
   <si>
     <t>HQ-raktar-printer</t>
@@ -163,12 +163,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -181,16 +187,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -207,10 +213,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -230,6 +236,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
@@ -429,12 +436,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -466,10 +473,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -708,12 +715,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1017,10 +1024,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1265,13 +1272,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.6719" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.6719" style="1" customWidth="1"/>
-    <col min="3" max="5" width="12.6719" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="12.6719" style="1" customWidth="1"/>
+    <col min="3" max="6" width="12.6719" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="12.6719" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
@@ -1280,6 +1287,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" s="2"/>
@@ -1287,6 +1295,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" ht="13.65" customHeight="1">
       <c r="A3" s="2"/>
@@ -1294,6 +1303,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
     </row>
     <row r="4" ht="13.65" customHeight="1">
       <c r="A4" s="2"/>
@@ -1301,28 +1311,31 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="3">
         <v>0</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" t="s" s="3">
+      <c r="C5" s="3"/>
+      <c r="D5" t="s" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="2"/>
       <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" t="s" s="3">
         <v>2</v>
       </c>
-      <c r="C6" t="s" s="3">
+      <c r="C6" s="3"/>
+      <c r="D6" t="s" s="3">
         <v>3</v>
       </c>
-      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" s="2"/>
@@ -1330,6 +1343,7 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" s="2"/>
@@ -1339,241 +1353,267 @@
       <c r="C8" t="s" s="3">
         <v>5</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" t="s" s="3">
+        <v>6</v>
+      </c>
       <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" t="s" s="3">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s" s="3">
         <v>7</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="C9" s="3"/>
+      <c r="D9" t="s" s="3">
+        <v>8</v>
+      </c>
       <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" s="2"/>
-      <c r="B10" t="s" s="3">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s" s="3">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
       <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" s="2"/>
       <c r="B11" t="s" s="3">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" t="s" s="3">
         <v>10</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" t="s" s="3">
-        <v>11</v>
-      </c>
       <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" t="s" s="3">
         <v>12</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" t="s" s="3">
-        <v>11</v>
-      </c>
-      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="B13" t="s" s="3">
+        <v>13</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="E13" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="F13" s="2"/>
     </row>
     <row r="14" ht="13.65" customHeight="1">
-      <c r="A14" t="s" s="3">
-        <v>13</v>
-      </c>
+      <c r="A14" s="2"/>
       <c r="B14" s="2"/>
-      <c r="C14" t="s" s="3">
-        <v>14</v>
-      </c>
-      <c r="D14" t="s" s="3">
-        <v>15</v>
-      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
       <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" s="2"/>
-      <c r="B15" t="s" s="3">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s" s="3">
-        <v>16</v>
-      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
     </row>
     <row r="16" ht="13.65" customHeight="1">
-      <c r="A16" s="2"/>
+      <c r="A16" t="s" s="3">
+        <v>14</v>
+      </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="C16" s="3"/>
+      <c r="D16" t="s" s="3">
+        <v>15</v>
+      </c>
+      <c r="E16" t="s" s="3">
+        <v>16</v>
+      </c>
+      <c r="F16" s="2"/>
     </row>
     <row r="17" ht="13.65" customHeight="1">
       <c r="A17" s="2"/>
       <c r="B17" t="s" s="3">
-        <v>4</v>
-      </c>
-      <c r="C17" t="s" s="3">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" t="s" s="3">
         <v>17</v>
       </c>
-      <c r="D17" s="2"/>
       <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
     </row>
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" s="2"/>
-      <c r="B18" t="s" s="3">
-        <v>18</v>
-      </c>
-      <c r="C18" t="s" s="3">
-        <v>19</v>
-      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" t="s" s="3">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C19" t="s" s="3">
-        <v>21</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="D19" t="s" s="3">
+        <v>19</v>
+      </c>
       <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
     </row>
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" s="2"/>
       <c r="B20" t="s" s="3">
-        <v>22</v>
-      </c>
-      <c r="C20" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="C20" s="3"/>
       <c r="D20" t="s" s="3">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
     </row>
     <row r="21" ht="13.65" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" t="s" s="3">
+        <v>22</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" t="s" s="3">
         <v>23</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" t="s" s="3">
-        <v>11</v>
-      </c>
       <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
     </row>
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
+      <c r="B22" t="s" s="3">
+        <v>24</v>
+      </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+      <c r="E22" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" ht="13.65" customHeight="1">
-      <c r="A23" t="s" s="3">
-        <v>24</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" t="s" s="3">
+      <c r="A23" s="2"/>
+      <c r="B23" t="s" s="3">
         <v>25</v>
       </c>
-      <c r="D23" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="E23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" ht="13.65" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" t="s" s="3">
-        <v>2</v>
-      </c>
-      <c r="C24" t="s" s="3">
-        <v>27</v>
-      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
     </row>
     <row r="25" ht="13.65" customHeight="1">
-      <c r="A25" s="2"/>
+      <c r="A25" t="s" s="3">
+        <v>26</v>
+      </c>
       <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
+      <c r="C25" s="3"/>
+      <c r="D25" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="E25" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="F25" s="2"/>
     </row>
     <row r="26" ht="13.65" customHeight="1">
       <c r="A26" s="2"/>
       <c r="B26" t="s" s="3">
-        <v>4</v>
-      </c>
-      <c r="C26" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="D26" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" t="s" s="3">
+        <v>29</v>
+      </c>
       <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
     </row>
     <row r="27" ht="13.65" customHeight="1">
       <c r="A27" s="2"/>
-      <c r="B27" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C27" t="s" s="3">
-        <v>30</v>
-      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
     </row>
     <row r="28" ht="13.65" customHeight="1">
       <c r="A28" s="2"/>
       <c r="B28" t="s" s="3">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="D28" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="D28" t="s" s="3">
+        <v>30</v>
+      </c>
       <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
     </row>
     <row r="29" ht="13.65" customHeight="1">
       <c r="A29" s="2"/>
-      <c r="B29" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" t="s" s="3">
-        <v>11</v>
-      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
       <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
     </row>
     <row r="30" ht="13.65" customHeight="1">
       <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="B30" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" t="s" s="3">
+        <v>32</v>
+      </c>
       <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
     </row>
     <row r="31" ht="13.65" customHeight="1">
       <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="B31" t="s" s="3">
+        <v>33</v>
+      </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
+      <c r="E31" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="F31" s="2"/>
     </row>
     <row r="32" ht="13.65" customHeight="1">
       <c r="A32" s="2"/>
@@ -1581,17 +1621,15 @@
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
     </row>
     <row r="33" ht="13.65" customHeight="1">
-      <c r="A33" t="s" s="3">
-        <v>34</v>
-      </c>
+      <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" t="s" s="3">
-        <v>35</v>
-      </c>
+      <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
     </row>
     <row r="34" ht="13.65" customHeight="1">
       <c r="A34" s="2"/>
@@ -1599,13 +1637,19 @@
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
     </row>
     <row r="35" ht="13.65" customHeight="1">
-      <c r="A35" s="2"/>
+      <c r="A35" t="s" s="3">
+        <v>34</v>
+      </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="C35" s="3"/>
+      <c r="D35" t="s" s="3">
+        <v>35</v>
+      </c>
       <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
     </row>
     <row r="36" ht="13.65" customHeight="1">
       <c r="A36" s="2"/>
@@ -1613,39 +1657,59 @@
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
     </row>
     <row r="37" ht="13.65" customHeight="1">
-      <c r="A37" t="s" s="3">
-        <v>36</v>
-      </c>
+      <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" t="s" s="3">
-        <v>37</v>
-      </c>
+      <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
     </row>
     <row r="38" ht="13.65" customHeight="1">
-      <c r="A38" t="s" s="3">
-        <v>38</v>
-      </c>
+      <c r="A38" s="2"/>
       <c r="B38" s="2"/>
-      <c r="C38" t="s" s="3">
-        <v>39</v>
-      </c>
+      <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
     </row>
     <row r="39" ht="13.65" customHeight="1">
       <c r="A39" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="3"/>
+      <c r="D39" t="s" s="3">
+        <v>37</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" ht="13.65" customHeight="1">
+      <c r="A40" t="s" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="3"/>
+      <c r="D40" t="s" s="3">
+        <v>39</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" ht="13.65" customHeight="1">
+      <c r="A41" t="s" s="3">
         <v>40</v>
       </c>
-      <c r="B39" s="2"/>
-      <c r="C39" t="s" s="3">
+      <c r="B41" s="2"/>
+      <c r="C41" s="3"/>
+      <c r="D41" t="s" s="3">
         <v>41</v>
       </c>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>

<commit_message>
További 2 telephely felkonfigolva
Elkészültem a Szigetvári és a Mohácsi telephely eszközkonfigjával.
Routereken statikus ip beállítva és a dhcp is. Switchek menedzsment beállítása is kész.

Létrehoztem két Rich text filet amibe mentettem a CLI parancsokat.

Pingeltem is és működött.
</commit_message>
<xml_diff>
--- a/IP terv.xlsx
+++ b/IP terv.xlsx
@@ -1,17 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zolta\Documents\GitHub\414\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E35BB2-15DE-4EBC-B5FA-FEC4293F73A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Munkalap1" sheetId="1" r:id="rId4"/>
+    <sheet name="Munkalap1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="62">
   <si>
     <t>Pécsi telephely LAN1 iroda</t>
   </si>
@@ -137,30 +151,77 @@
   </si>
   <si>
     <t>10.10.30.0/30</t>
+  </si>
+  <si>
+    <t>Mohácsi telephely LAN (bolt)</t>
+  </si>
+  <si>
+    <t>192.168.21.0/24</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>SW21</t>
+  </si>
+  <si>
+    <t>SW31</t>
+  </si>
+  <si>
+    <t>192.168.31.11-100</t>
+  </si>
+  <si>
+    <t>Sziget-bolt-printer</t>
+  </si>
+  <si>
+    <t>Sziget-bolt-PC1</t>
+  </si>
+  <si>
+    <t>Sziget-bolt-PC2</t>
+  </si>
+  <si>
+    <t>192.168.31.1</t>
+  </si>
+  <si>
+    <t>192.168.31.2</t>
+  </si>
+  <si>
+    <t>192.168.31.10</t>
+  </si>
+  <si>
+    <t>192.168.21.11-100</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>192.168.21.1</t>
+  </si>
+  <si>
+    <t>192.168.21.2</t>
+  </si>
+  <si>
+    <t>Moha-bolt-printer</t>
+  </si>
+  <si>
+    <t>Moha-bolt-PC1</t>
+  </si>
+  <si>
+    <t>Moha-bolt-PC2</t>
+  </si>
+  <si>
+    <t>192.168.21.10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -187,64 +248,117 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
+        <color theme="9" tint="-0.249977111117893"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color theme="9" tint="-0.249977111117893"/>
       </right>
       <top style="thin">
-        <color indexed="10"/>
+        <color theme="9" tint="-0.249977111117893"/>
       </top>
       <bottom style="thin">
-        <color indexed="10"/>
+        <color theme="9" tint="-0.249977111117893"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -446,7 +560,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -464,7 +578,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -493,7 +607,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -518,7 +632,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -543,7 +657,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -568,7 +682,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -593,7 +707,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -618,7 +732,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -643,7 +757,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -668,7 +782,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -693,7 +807,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -706,9 +820,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -725,7 +845,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -743,7 +863,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -768,7 +888,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -793,7 +913,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -818,7 +938,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -843,7 +963,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -868,7 +988,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -893,7 +1013,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -918,7 +1038,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -943,7 +1063,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -968,7 +1088,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -981,9 +1101,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -997,7 +1123,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1015,7 +1141,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1044,7 +1170,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1069,7 +1195,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1094,7 +1220,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1119,7 +1245,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1144,7 +1270,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1169,7 +1295,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1194,7 +1320,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1219,7 +1345,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1244,7 +1370,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1257,409 +1383,422 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F59"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6719" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6719" style="1" customWidth="1"/>
-    <col min="3" max="6" width="12.6719" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="12.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.6640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="12.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.65" customHeight="1">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2" ht="13.65" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" ht="13.65" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" ht="13.65" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" ht="13.65" customHeight="1">
-      <c r="A5" t="s" s="3">
+    <row r="1" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" t="s" s="3">
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" ht="13.65" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" t="s" s="3">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" t="s" s="3">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" ht="13.65" customHeight="1">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" ht="13.65" customHeight="1">
-      <c r="A8" s="2"/>
-      <c r="B8" t="s" s="3">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C8" t="s" s="3">
+      <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D8" t="s" s="3">
+      <c r="D8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" ht="13.65" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" t="s" s="3">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" t="s" s="3">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" ht="13.65" customHeight="1">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" ht="13.65" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" t="s" s="3">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" t="s" s="3">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" ht="13.65" customHeight="1">
-      <c r="A12" s="2"/>
-      <c r="B12" t="s" s="3">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" t="s" s="3">
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" ht="13.65" customHeight="1">
-      <c r="A13" s="2"/>
-      <c r="B13" t="s" s="3">
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" t="s" s="3">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" ht="13.65" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" ht="13.65" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" ht="13.65" customHeight="1">
-      <c r="A16" t="s" s="3">
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" t="s" s="3">
+      <c r="B16" s="3"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E16" t="s" s="3">
+      <c r="E16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" ht="13.65" customHeight="1">
-      <c r="A17" s="2"/>
-      <c r="B17" t="s" s="3">
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C17" s="3"/>
-      <c r="D17" t="s" s="3">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" ht="13.65" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" ht="13.65" customHeight="1">
-      <c r="A19" s="2"/>
-      <c r="B19" t="s" s="3">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C19" t="s" s="3">
+      <c r="C19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D19" t="s" s="3">
+      <c r="D19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" ht="13.65" customHeight="1">
-      <c r="A20" s="2"/>
-      <c r="B20" t="s" s="3">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" t="s" s="3">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" ht="13.65" customHeight="1">
-      <c r="A21" s="2"/>
-      <c r="B21" t="s" s="3">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" t="s" s="3">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" ht="13.65" customHeight="1">
-      <c r="A22" s="2"/>
-      <c r="B22" t="s" s="3">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" t="s" s="3">
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" ht="13.65" customHeight="1">
-      <c r="A23" s="2"/>
-      <c r="B23" t="s" s="3">
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" t="s" s="3">
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" ht="13.65" customHeight="1">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" ht="13.65" customHeight="1">
-      <c r="A25" t="s" s="3">
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" t="s" s="3">
+      <c r="B25" s="3"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E25" t="s" s="3">
+      <c r="E25" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" ht="13.65" customHeight="1">
-      <c r="A26" s="2"/>
-      <c r="B26" t="s" s="3">
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="3"/>
-      <c r="D26" t="s" s="3">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" ht="13.65" customHeight="1">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-    </row>
-    <row r="28" ht="13.65" customHeight="1">
-      <c r="A28" s="2"/>
-      <c r="B28" t="s" s="3">
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+    </row>
+    <row r="27" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C28" t="s" s="3">
+      <c r="C28" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D28" t="s" s="3">
+      <c r="D28" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-    </row>
-    <row r="29" ht="13.65" customHeight="1">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" ht="13.65" customHeight="1">
-      <c r="A30" s="2"/>
-      <c r="B30" t="s" s="3">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="29" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+    </row>
+    <row r="30" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C30" s="3"/>
-      <c r="D30" t="s" s="3">
+      <c r="C30" s="4"/>
+      <c r="D30" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="31" ht="13.65" customHeight="1">
-      <c r="A31" s="2"/>
-      <c r="B31" t="s" s="3">
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+    </row>
+    <row r="31" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" t="s" s="3">
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F31" s="2"/>
-    </row>
-    <row r="32" ht="13.65" customHeight="1">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" ht="13.65" customHeight="1">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" ht="13.65" customHeight="1">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" ht="13.65" customHeight="1">
-      <c r="A35" t="s" s="3">
+      <c r="F31" s="3"/>
+    </row>
+    <row r="32" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+    </row>
+    <row r="33" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+    </row>
+    <row r="34" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+    </row>
+    <row r="35" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="3"/>
-      <c r="D35" t="s" s="3">
+      <c r="B35" s="3"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" ht="13.65" customHeight="1">
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+    </row>
+    <row r="36" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
+      <c r="B36" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="D36" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" ht="13.65" customHeight="1">
+    <row r="37" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1667,53 +1806,249 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" ht="13.65" customHeight="1">
+    <row r="38" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="B38" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" ht="13.65" customHeight="1">
-      <c r="A39" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="3"/>
-      <c r="D39" t="s" s="3">
-        <v>37</v>
+    <row r="39" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" ht="13.65" customHeight="1">
-      <c r="A40" t="s" s="3">
-        <v>38</v>
-      </c>
+    <row r="40" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="3"/>
-      <c r="D40" t="s" s="3">
-        <v>39</v>
-      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" ht="13.65" customHeight="1">
-      <c r="A41" t="s" s="3">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2"/>
-      <c r="C41" s="3"/>
-      <c r="D41" t="s" s="3">
-        <v>41</v>
+    <row r="41" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
     </row>
+    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+    </row>
+    <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+    </row>
+    <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+    </row>
+    <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+    </row>
+    <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+    </row>
+    <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+    </row>
+    <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F53" s="3"/>
+    </row>
+    <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+    </row>
+    <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B57" s="3"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+    </row>
+    <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B58" s="3"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+    </row>
+    <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B59" s="3"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
hq atazervezes, szerver telepites
Atszerveztem a HQ topologiat, R1 G0/0 felszabaditva ASA es WAN csatlakoztatasra
CoreSW beszerelve
G0/1 a LAN oldal
VLAN10 mgmt-szerver
VLAN11 iroda
VLAN12 bolt
VLAN13 raktar

a trunk portokon VLAN10-13 engedve.
SW11-SW12 osszekotve L2 tartalek celbol
Core sw az STP root primary, masi ketto root secondary

A szerver ip cime 192.168.10.20 DNS funkciot lat el, felvettem par static DNS rekordot (nyomtatok)

.rtf konfig fajlok torolve, helyette a PT startup config/export funkciojaval mentett fajl kerul fel.
</commit_message>
<xml_diff>
--- a/IP terv.xlsx
+++ b/IP terv.xlsx
@@ -1,31 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zolta\Documents\GitHub\414\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E35BB2-15DE-4EBC-B5FA-FEC4293F73A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <bookViews>
-    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="Munkalap1" sheetId="1" r:id="rId1"/>
+    <sheet name="Munkalap1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="50">
+  <si>
+    <t>Pécsi telephely mgmt - szerverek</t>
+  </si>
+  <si>
+    <t>192.168.10.0/24</t>
+  </si>
+  <si>
+    <t>VLAN10</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>G0/1</t>
+  </si>
+  <si>
+    <t>192.168.10.1</t>
+  </si>
+  <si>
+    <t>SW10</t>
+  </si>
+  <si>
+    <t>192.168.10.10</t>
+  </si>
+  <si>
+    <t>SW11</t>
+  </si>
+  <si>
+    <t>192.168.10.11</t>
+  </si>
+  <si>
+    <t>SW12</t>
+  </si>
+  <si>
+    <t>192.168.10.12</t>
+  </si>
+  <si>
+    <t>DNS szerver</t>
+  </si>
+  <si>
+    <t>129.168.10.20</t>
+  </si>
   <si>
     <t>Pécsi telephely LAN1 iroda</t>
   </si>
@@ -33,27 +61,18 @@
     <t>192.168.11.0/24</t>
   </si>
   <si>
+    <t>VLAN11</t>
+  </si>
+  <si>
     <t>DHCP tartomány</t>
   </si>
   <si>
     <t>192.168.11.11-100</t>
   </si>
   <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>G0/0</t>
-  </si>
-  <si>
     <t>192.168.11.1</t>
   </si>
   <si>
-    <t>SW11</t>
-  </si>
-  <si>
-    <t>192.168.11.2</t>
-  </si>
-  <si>
     <t>HQ-iroda-printer</t>
   </si>
   <si>
@@ -81,18 +100,9 @@
     <t>192.168.12.11-100</t>
   </si>
   <si>
-    <t>G0/1</t>
-  </si>
-  <si>
     <t>192.168.12.1</t>
   </si>
   <si>
-    <t>SW12</t>
-  </si>
-  <si>
-    <t>192.168.12.2</t>
-  </si>
-  <si>
     <t>HQ-bolt-printer</t>
   </si>
   <si>
@@ -151,77 +161,30 @@
   </si>
   <si>
     <t>10.10.30.0/30</t>
-  </si>
-  <si>
-    <t>Mohácsi telephely LAN (bolt)</t>
-  </si>
-  <si>
-    <t>192.168.21.0/24</t>
-  </si>
-  <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>SW21</t>
-  </si>
-  <si>
-    <t>SW31</t>
-  </si>
-  <si>
-    <t>192.168.31.11-100</t>
-  </si>
-  <si>
-    <t>Sziget-bolt-printer</t>
-  </si>
-  <si>
-    <t>Sziget-bolt-PC1</t>
-  </si>
-  <si>
-    <t>Sziget-bolt-PC2</t>
-  </si>
-  <si>
-    <t>192.168.31.1</t>
-  </si>
-  <si>
-    <t>192.168.31.2</t>
-  </si>
-  <si>
-    <t>192.168.31.10</t>
-  </si>
-  <si>
-    <t>192.168.21.11-100</t>
-  </si>
-  <si>
-    <t>R2</t>
-  </si>
-  <si>
-    <t>192.168.21.1</t>
-  </si>
-  <si>
-    <t>192.168.21.2</t>
-  </si>
-  <si>
-    <t>Moha-bolt-printer</t>
-  </si>
-  <si>
-    <t>Moha-bolt-PC1</t>
-  </si>
-  <si>
-    <t>Moha-bolt-PC2</t>
-  </si>
-  <si>
-    <t>192.168.21.10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="0" formatCode="General"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -248,117 +211,64 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="9" tint="-0.249977111117893"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color theme="9" tint="-0.249977111117893"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color theme="9" tint="-0.249977111117893"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color theme="9" tint="-0.249977111117893"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFAAAAAA"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
+      <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="ffff0000"/>
+      <rgbColor rgb="ff00ff00"/>
+      <rgbColor rgb="ff0000ff"/>
+      <rgbColor rgb="ffffff00"/>
+      <rgbColor rgb="ffff00ff"/>
+      <rgbColor rgb="ff00ffff"/>
+      <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -560,7 +470,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -578,7 +488,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -607,7 +517,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -632,7 +542,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -657,7 +567,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -682,7 +592,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -707,7 +617,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -732,7 +642,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -757,7 +667,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -782,7 +692,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -807,7 +717,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -820,15 +730,9 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -845,7 +749,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -863,7 +767,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -888,7 +792,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -913,7 +817,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -938,7 +842,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -963,7 +867,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -988,7 +892,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1013,7 +917,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1038,7 +942,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1063,7 +967,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1088,7 +992,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1101,15 +1005,9 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1123,7 +1021,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1141,7 +1039,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1170,7 +1068,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1195,7 +1093,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1220,7 +1118,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1245,7 +1143,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1270,7 +1168,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1295,7 +1193,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1320,7 +1218,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1345,7 +1243,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1370,7 +1268,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1383,422 +1281,427 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F45"/>
+  <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.6640625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="12.6640625" style="1"/>
+    <col min="1" max="1" width="12.6719" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6719" style="1" customWidth="1"/>
+    <col min="3" max="6" width="12.6719" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="12.6719" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="1" ht="13.65" customHeight="1">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" ht="13.65" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" ht="13.65" customHeight="1">
+      <c r="A3" t="s" s="3">
         <v>0</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" t="s" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E3" t="s" s="3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" ht="13.65" customHeight="1">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" ht="13.65" customHeight="1">
+      <c r="A5" s="3"/>
+      <c r="B5" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s" s="3">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s" s="3">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" ht="13.65" customHeight="1">
       <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s" s="3">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" t="s" s="3">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" ht="13.65" customHeight="1">
       <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
+      <c r="B7" t="s" s="3">
+        <v>8</v>
+      </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" t="s" s="3">
+        <v>9</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" ht="13.65" customHeight="1">
       <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s" s="3">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" ht="13.65" customHeight="1">
       <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" t="s" s="3">
+        <v>13</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" ht="13.65" customHeight="1">
       <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="2"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" ht="13.65" customHeight="1">
       <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" ht="13.65" customHeight="1">
       <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="B12" s="2"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" ht="13.65" customHeight="1">
+      <c r="A13" t="s" s="3">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="D13" t="s" s="3">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s" s="3">
+        <v>16</v>
+      </c>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" ht="13.65" customHeight="1">
+      <c r="A14" s="2"/>
+      <c r="B14" t="s" s="3">
+        <v>17</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="3"/>
-    </row>
-    <row r="17" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4" t="s">
+      <c r="D14" t="s" s="3">
+        <v>18</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" ht="13.65" customHeight="1">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" ht="13.65" customHeight="1">
+      <c r="A16" s="2"/>
+      <c r="B16" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s" s="3">
+        <v>4</v>
+      </c>
+      <c r="D16" t="s" s="3">
+        <v>19</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" ht="13.65" customHeight="1">
+      <c r="A17" s="2"/>
+      <c r="B17" t="s" s="3">
+        <v>20</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" t="s" s="3">
+        <v>21</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" ht="13.65" customHeight="1">
+      <c r="A18" s="2"/>
+      <c r="B18" t="s" s="3">
+        <v>22</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" ht="13.65" customHeight="1">
+      <c r="A19" s="2"/>
+      <c r="B19" t="s" s="3">
+        <v>24</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" ht="13.65" customHeight="1">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" ht="13.65" customHeight="1">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" ht="13.65" customHeight="1">
+      <c r="A22" t="s" s="3">
+        <v>25</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="3"/>
+      <c r="D22" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="E22" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F22" s="2"/>
+    </row>
+    <row r="23" ht="13.65" customHeight="1">
+      <c r="A23" s="2"/>
+      <c r="B23" t="s" s="3">
         <v>17</v>
       </c>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-    </row>
-    <row r="18" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-    </row>
-    <row r="19" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4" t="s">
+      <c r="C23" s="3"/>
+      <c r="D23" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" ht="13.65" customHeight="1">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" ht="13.65" customHeight="1">
+      <c r="A25" s="2"/>
+      <c r="B25" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s" s="3">
         <v>4</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-    </row>
-    <row r="20" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-    </row>
-    <row r="21" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4" t="s">
+      <c r="D25" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" ht="13.65" customHeight="1">
+      <c r="A26" s="2"/>
+      <c r="B26" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" ht="13.65" customHeight="1">
+      <c r="A27" s="2"/>
+      <c r="B27" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" t="s" s="3">
         <v>23</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-    </row>
-    <row r="22" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" s="3"/>
-    </row>
-    <row r="24" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-    </row>
-    <row r="25" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" s="3"/>
-    </row>
-    <row r="26" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-    </row>
-    <row r="27" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-    </row>
-    <row r="28" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="4" t="s">
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" ht="13.65" customHeight="1">
+      <c r="A28" s="2"/>
+      <c r="B28" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" ht="13.65" customHeight="1">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" ht="13.65" customHeight="1">
+      <c r="A30" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" s="3"/>
+      <c r="D30" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="E30" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="F30" s="2"/>
+    </row>
+    <row r="31" ht="13.65" customHeight="1">
+      <c r="A31" s="2"/>
+      <c r="B31" t="s" s="3">
+        <v>17</v>
+      </c>
+      <c r="C31" s="3"/>
+      <c r="D31" t="s" s="3">
+        <v>37</v>
+      </c>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="32" ht="13.65" customHeight="1">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" ht="13.65" customHeight="1">
+      <c r="A33" s="2"/>
+      <c r="B33" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s" s="3">
         <v>4</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-    </row>
-    <row r="29" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-    </row>
-    <row r="30" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-    </row>
-    <row r="31" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-    </row>
-    <row r="34" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
+      <c r="D33" t="s" s="3">
+        <v>38</v>
+      </c>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" ht="13.65" customHeight="1">
+      <c r="A34" s="2"/>
+      <c r="B34" t="s" s="3">
+        <v>39</v>
+      </c>
       <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-    </row>
-    <row r="35" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-    </row>
-    <row r="36" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D34" t="s" s="3">
+        <v>40</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+    </row>
+    <row r="35" ht="13.65" customHeight="1">
+      <c r="A35" s="2"/>
+      <c r="B35" t="s" s="3">
+        <v>41</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" ht="13.65" customHeight="1">
       <c r="A36" s="2"/>
-      <c r="B36" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" ht="13.65" customHeight="1">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1806,33 +1709,27 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" ht="13.65" customHeight="1">
       <c r="A38" s="2"/>
-      <c r="B38" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2" t="s">
-        <v>52</v>
+    <row r="39" ht="13.65" customHeight="1">
+      <c r="A39" t="s" s="3">
+        <v>42</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="3"/>
+      <c r="D39" t="s" s="3">
+        <v>43</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" ht="13.65" customHeight="1">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1840,215 +1737,61 @@
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="13.65" customHeight="1">
       <c r="A41" s="2"/>
-      <c r="B41" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="B41" s="2"/>
       <c r="C41" s="2"/>
-      <c r="D41" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
     </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" ht="13.65" customHeight="1">
       <c r="A42" s="2"/>
-      <c r="B42" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="E42" s="2"/>
       <c r="F42" s="2"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2" t="s">
-        <v>12</v>
-      </c>
+    <row r="43" ht="13.65" customHeight="1">
+      <c r="A43" t="s" s="3">
+        <v>44</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" s="3"/>
+      <c r="D43" t="s" s="3">
+        <v>45</v>
+      </c>
+      <c r="E43" s="2"/>
       <c r="F43" s="2"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2"/>
+    <row r="44" ht="13.65" customHeight="1">
+      <c r="A44" t="s" s="3">
+        <v>46</v>
+      </c>
       <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
+      <c r="C44" s="3"/>
+      <c r="D44" t="s" s="3">
+        <v>47</v>
+      </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
     </row>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2"/>
+    <row r="45" ht="13.65" customHeight="1">
+      <c r="A45" t="s" s="3">
+        <v>48</v>
+      </c>
       <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
+      <c r="C45" s="3"/>
+      <c r="D45" t="s" s="3">
+        <v>49</v>
+      </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
     </row>
-    <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-    </row>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-    </row>
-    <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-    </row>
-    <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-    </row>
-    <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-    </row>
-    <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F53" s="3"/>
-    </row>
-    <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-    </row>
-    <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B57" s="3"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-    </row>
-    <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="3"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-    </row>
-    <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B59" s="3"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
IP terv .xlsx fájl bővítése
R2 és R3  IP konfigjával bővítettem a .xlsx fájlt

Jirában készre jelöltem a ticketeket.
</commit_message>
<xml_diff>
--- a/IP terv.xlsx
+++ b/IP terv.xlsx
@@ -1,17 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zolta\Documents\GitHub\414\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C93E105-AA62-4549-9137-9E62D72122AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Munkalap1" sheetId="1" r:id="rId4"/>
+    <sheet name="Munkalap1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="90">
   <si>
     <t>Pécsi telephely mgmt - szerverek</t>
   </si>
@@ -221,30 +235,77 @@
   </si>
   <si>
     <t>203.0.113.3/24</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>G0/0</t>
+  </si>
+  <si>
+    <t>192.168.21.11-100</t>
+  </si>
+  <si>
+    <t>192.168.21.1</t>
+  </si>
+  <si>
+    <t>mohács-bolt-printer</t>
+  </si>
+  <si>
+    <t>mohács-bolt-PC1</t>
+  </si>
+  <si>
+    <t>mohács-bolt-PC2</t>
+  </si>
+  <si>
+    <t>192.168.21.10</t>
+  </si>
+  <si>
+    <t>SW21</t>
+  </si>
+  <si>
+    <t>VLAN 1</t>
+  </si>
+  <si>
+    <t>192.168.21.2</t>
+  </si>
+  <si>
+    <t>192.168.31.11-100</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>192.168.31.1</t>
+  </si>
+  <si>
+    <t>SW31</t>
+  </si>
+  <si>
+    <t>192.168.31.2</t>
+  </si>
+  <si>
+    <t>szigetvár-bolt-printer</t>
+  </si>
+  <si>
+    <t>szigetvár-bolt-PC1</t>
+  </si>
+  <si>
+    <t>szigetvár-bolt-PC2</t>
+  </si>
+  <si>
+    <t>192.168.31.10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -261,7 +322,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -284,51 +345,114 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -530,7 +654,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -548,7 +672,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -577,7 +701,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -602,7 +726,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -627,7 +751,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -652,7 +776,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -677,7 +801,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -702,7 +826,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -727,7 +851,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -752,7 +876,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -777,7 +901,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -790,9 +914,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -809,7 +939,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -827,7 +957,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -852,7 +982,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -877,7 +1007,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -902,7 +1032,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -927,7 +1057,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -952,7 +1082,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -977,7 +1107,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1002,7 +1132,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1027,7 +1157,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1052,7 +1182,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1065,9 +1195,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1081,7 +1217,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1099,7 +1235,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1128,7 +1264,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1153,7 +1289,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1178,7 +1314,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1203,7 +1339,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1228,7 +1364,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1253,7 +1389,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1278,7 +1414,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1303,7 +1439,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1328,7 +1464,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1341,31 +1477,40 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
-  <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F67"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6719" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6719" style="1" customWidth="1"/>
-    <col min="3" max="6" width="12.6719" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="12.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.6640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="12.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.65" customHeight="1">
+    <row r="1" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1373,7 +1518,7 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" ht="13.65" customHeight="1">
+    <row r="2" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1381,21 +1526,21 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" ht="13.65" customHeight="1">
-      <c r="A3" t="s" s="3">
+    <row r="3" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" t="s" s="3">
+      <c r="D3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" t="s" s="3">
+      <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" ht="13.65" customHeight="1">
+    <row r="4" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1403,83 +1548,83 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" ht="13.65" customHeight="1">
+    <row r="5" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
-      <c r="B5" t="s" s="3">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="s" s="3">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" t="s" s="3">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" ht="13.65" customHeight="1">
+    <row r="6" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
-      <c r="B6" t="s" s="3">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" t="s" s="3">
+      <c r="D6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" ht="13.65" customHeight="1">
+    <row r="7" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
-      <c r="B7" t="s" s="3">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" t="s" s="3">
+      <c r="D7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" ht="13.65" customHeight="1">
+    <row r="8" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
-      <c r="B8" t="s" s="3">
+      <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" t="s" s="3">
+      <c r="D8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" ht="13.65" customHeight="1">
+    <row r="9" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="B9" t="s" s="3">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" t="s" s="3">
+      <c r="D9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" t="s" s="3">
+      <c r="F9" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" ht="13.65" customHeight="1">
+    <row r="10" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
-      <c r="B10" t="s" s="3">
+      <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="3"/>
-      <c r="D10" t="s" s="3">
+      <c r="D10" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" ht="13.65" customHeight="1">
+    <row r="11" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="2"/>
       <c r="C11" s="3"/>
@@ -1487,7 +1632,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" ht="13.65" customHeight="1">
+    <row r="12" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
@@ -1495,33 +1640,33 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" ht="13.65" customHeight="1">
-      <c r="A13" t="s" s="3">
+    <row r="13" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="3"/>
-      <c r="D13" t="s" s="3">
+      <c r="D13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E13" t="s" s="3">
+      <c r="E13" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" ht="13.65" customHeight="1">
+    <row r="14" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" t="s" s="3">
+      <c r="B14" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" t="s" s="3">
+      <c r="D14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" ht="13.65" customHeight="1">
+    <row r="15" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1529,57 +1674,57 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" ht="13.65" customHeight="1">
+    <row r="16" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" t="s" s="3">
+      <c r="B16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C16" t="s" s="3">
+      <c r="C16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D16" t="s" s="3">
+      <c r="D16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" ht="13.65" customHeight="1">
+    <row r="17" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" t="s" s="3">
+      <c r="B17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="3"/>
-      <c r="D17" t="s" s="3">
+      <c r="D17" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" ht="13.65" customHeight="1">
+    <row r="18" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" t="s" s="3">
+      <c r="B18" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" t="s" s="3">
+      <c r="E18" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" ht="13.65" customHeight="1">
+    <row r="19" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" t="s" s="3">
+      <c r="B19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" t="s" s="3">
+      <c r="E19" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" ht="13.65" customHeight="1">
+    <row r="20" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1587,7 +1732,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" ht="13.65" customHeight="1">
+    <row r="21" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1595,33 +1740,33 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" ht="13.65" customHeight="1">
-      <c r="A22" t="s" s="3">
+    <row r="22" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="3"/>
-      <c r="D22" t="s" s="3">
+      <c r="D22" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E22" t="s" s="3">
+      <c r="E22" s="3" t="s">
         <v>30</v>
       </c>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" ht="13.65" customHeight="1">
+    <row r="23" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" t="s" s="3">
+      <c r="B23" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C23" s="3"/>
-      <c r="D23" t="s" s="3">
+      <c r="D23" s="3" t="s">
         <v>31</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" ht="13.65" customHeight="1">
+    <row r="24" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1629,57 +1774,57 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" ht="13.65" customHeight="1">
+    <row r="25" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" t="s" s="3">
+      <c r="B25" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C25" t="s" s="3">
+      <c r="C25" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D25" t="s" s="3">
+      <c r="D25" s="3" t="s">
         <v>32</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" ht="13.65" customHeight="1">
+    <row r="26" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" t="s" s="3">
+      <c r="B26" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C26" s="3"/>
-      <c r="D26" t="s" s="3">
+      <c r="D26" s="3" t="s">
         <v>34</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" ht="13.65" customHeight="1">
+    <row r="27" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" t="s" s="3">
+      <c r="B27" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" t="s" s="3">
+      <c r="E27" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" ht="13.65" customHeight="1">
+    <row r="28" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" t="s" s="3">
+      <c r="B28" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
-      <c r="E28" t="s" s="3">
+      <c r="E28" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" ht="13.65" customHeight="1">
+    <row r="29" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1687,33 +1832,33 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" ht="13.65" customHeight="1">
-      <c r="A30" t="s" s="3">
+    <row r="30" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="3"/>
-      <c r="D30" t="s" s="3">
+      <c r="D30" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E30" t="s" s="3">
+      <c r="E30" s="3" t="s">
         <v>39</v>
       </c>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" ht="13.65" customHeight="1">
+    <row r="31" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" t="s" s="3">
+      <c r="B31" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="3"/>
-      <c r="D31" t="s" s="3">
+      <c r="D31" s="3" t="s">
         <v>40</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" ht="13.65" customHeight="1">
+    <row r="32" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1721,45 +1866,45 @@
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
     </row>
-    <row r="33" ht="13.65" customHeight="1">
+    <row r="33" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" t="s" s="3">
+      <c r="B33" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C33" t="s" s="3">
+      <c r="C33" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D33" t="s" s="3">
+      <c r="D33" s="3" t="s">
         <v>41</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" ht="13.65" customHeight="1">
+    <row r="34" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
-      <c r="B34" t="s" s="3">
+      <c r="B34" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="3"/>
-      <c r="D34" t="s" s="3">
+      <c r="D34" s="3" t="s">
         <v>43</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" ht="13.65" customHeight="1">
+    <row r="35" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" t="s" s="3">
+      <c r="B35" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
-      <c r="E35" t="s" s="3">
+      <c r="E35" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" ht="13.65" customHeight="1">
+    <row r="36" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1767,27 +1912,31 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" ht="13.65" customHeight="1">
-      <c r="A37" t="s" s="3">
+    <row r="37" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" t="s" s="3">
+      <c r="D37" s="3" t="s">
         <v>46</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" ht="13.65" customHeight="1">
+    <row r="38" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
+      <c r="B38" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="D38" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" ht="13.65" customHeight="1">
+    <row r="39" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="2"/>
       <c r="C39" s="3"/>
@@ -1795,217 +1944,333 @@
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" ht="13.65" customHeight="1">
+    <row r="40" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
+      <c r="B40" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" ht="13.65" customHeight="1">
+    <row r="41" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
-      <c r="B41" s="2"/>
+      <c r="B41" s="1" t="s">
+        <v>78</v>
+      </c>
       <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="2"/>
+      <c r="D41" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="F41" s="2"/>
     </row>
-    <row r="42" ht="13.65" customHeight="1">
-      <c r="A42" t="s" s="3">
-        <v>47</v>
-      </c>
-      <c r="B42" s="2"/>
+    <row r="42" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="C42" s="3"/>
-      <c r="D42" t="s" s="3">
-        <v>48</v>
-      </c>
-      <c r="E42" s="2"/>
+      <c r="D42" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F42" s="2"/>
     </row>
-    <row r="43" ht="13.65" customHeight="1">
+    <row r="43" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
-      <c r="B43" s="2"/>
+      <c r="B43" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
-      <c r="E43" s="2"/>
+      <c r="E43" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F43" s="2"/>
     </row>
-    <row r="44" ht="13.65" customHeight="1">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
+    <row r="44" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3"/>
+      <c r="B44" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
     </row>
-    <row r="45" ht="13.65" customHeight="1">
-      <c r="A45" s="2"/>
+    <row r="45" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
     </row>
-    <row r="46" ht="13.65" customHeight="1">
-      <c r="A46" s="2"/>
+    <row r="46" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
     </row>
-    <row r="47" ht="13.65" customHeight="1">
-      <c r="A47" t="s" s="3">
-        <v>49</v>
-      </c>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" t="s" s="3">
-        <v>50</v>
+    <row r="47" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3"/>
+      <c r="B47" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
-    <row r="48" ht="13.65" customHeight="1">
-      <c r="A48" s="2"/>
-      <c r="B48" t="s" s="3">
-        <v>51</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" t="s" s="3">
-        <v>52</v>
-      </c>
+    <row r="48" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
-    <row r="49" ht="13.65" customHeight="1">
-      <c r="A49" s="2"/>
-      <c r="B49" t="s" s="3">
-        <v>53</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" t="s" s="3">
-        <v>26</v>
-      </c>
+    <row r="49" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3"/>
+      <c r="B49" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
-    <row r="50" ht="13.65" customHeight="1">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
+    <row r="50" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3"/>
+      <c r="B50" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="F50" s="2"/>
     </row>
-    <row r="51" ht="13.65" customHeight="1">
-      <c r="A51" t="s" s="3">
-        <v>54</v>
-      </c>
-      <c r="B51" s="2"/>
-      <c r="C51" t="s" s="3">
-        <v>55</v>
-      </c>
-      <c r="D51" t="s" s="3">
-        <v>56</v>
+    <row r="51" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
-    <row r="52" ht="13.65" customHeight="1">
-      <c r="A52" t="s" s="3">
-        <v>57</v>
-      </c>
-      <c r="B52" s="2"/>
-      <c r="C52" t="s" s="3">
-        <v>58</v>
-      </c>
-      <c r="D52" t="s" s="3">
-        <v>59</v>
-      </c>
-      <c r="E52" s="2"/>
+    <row r="52" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F52" s="2"/>
     </row>
-    <row r="53" ht="13.65" customHeight="1">
-      <c r="A53" t="s" s="3">
-        <v>60</v>
-      </c>
-      <c r="B53" s="2"/>
-      <c r="C53" t="s" s="3">
-        <v>61</v>
-      </c>
-      <c r="D53" t="s" s="3">
-        <v>62</v>
-      </c>
-      <c r="E53" s="2"/>
+    <row r="53" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F53" s="2"/>
     </row>
-    <row r="54" ht="13.65" customHeight="1">
-      <c r="A54" t="s" s="3">
-        <v>63</v>
-      </c>
+    <row r="54" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
       <c r="B54" s="2"/>
-      <c r="C54" t="s" s="3">
-        <v>64</v>
-      </c>
-      <c r="D54" t="s" s="3">
-        <v>65</v>
-      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
     </row>
-    <row r="55" ht="13.65" customHeight="1">
-      <c r="A55" s="3"/>
+    <row r="55" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="B55" s="2"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
     </row>
-    <row r="56" ht="13.65" customHeight="1">
-      <c r="A56" t="s" s="3">
-        <v>66</v>
-      </c>
-      <c r="B56" s="2"/>
-      <c r="C56" s="3"/>
-      <c r="D56" t="s" s="3">
-        <v>67</v>
+    <row r="56" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
     </row>
-    <row r="57" ht="13.65" customHeight="1">
-      <c r="A57" t="s" s="3">
-        <v>68</v>
-      </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="3"/>
-      <c r="D57" t="s" s="3">
-        <v>69</v>
-      </c>
-      <c r="E57" s="2"/>
+    <row r="57" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="F57" s="2"/>
     </row>
-    <row r="58" ht="13.65" customHeight="1">
-      <c r="A58" s="3"/>
+    <row r="58" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
-    <row r="59" ht="13.65" customHeight="1">
-      <c r="A59" s="3"/>
+    <row r="59" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="B59" s="2"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
+      <c r="C59" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
     </row>
+    <row r="60" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+    </row>
+    <row r="61" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+    </row>
+    <row r="62" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B62" s="2"/>
+      <c r="C62" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+    </row>
+    <row r="64" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="2"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="65" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B65" s="2"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+    </row>
+    <row r="66" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="3"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+    </row>
+    <row r="67" spans="1:6" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="3"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>